<commit_message>
chore: 달란트 일일 백업 (2026-09-16)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="2026-09-15" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="2026-09-16" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="156">
   <si>
     <t>이름</t>
   </si>
@@ -3352,6 +3353,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>477</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>367</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>377</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>20</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>114</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>74</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>179</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>84</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>66</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>187</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39">
+        <v>20</v>
+      </c>
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42" t="s">
+        <v>68</v>
+      </c>
+      <c r="D42">
+        <v>30</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43">
+        <v>23</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44">
+        <v>59</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45">
+        <v>3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>73</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47">
+        <v>26</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>74</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48">
+        <v>20</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49">
+        <v>3</v>
+      </c>
+      <c r="C49" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>78</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52">
+        <v>54</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>80</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>81</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>82</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>48</v>
+      </c>
+      <c r="D55">
+        <v>154</v>
+      </c>
+      <c r="E55" t="s">
+        <v>83</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>59</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>20</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>235</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>86</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>20</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>203</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>349</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>171</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>229</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>161</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>38</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>29</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>3</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>187</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>195</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>387</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>46</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>20</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>47</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>105</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>545</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>139</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>187</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>20</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>46</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>33</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>23</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>3</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-17)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -6,13 +6,14 @@
   <sheets>
     <sheet sheetId="1" name="2026-09-15" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="2026-09-16" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="2026-09-17" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="156">
   <si>
     <t>이름</t>
   </si>
@@ -5852,6 +5853,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>730</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>570</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>600</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>267</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>74</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>179</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>84</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>66</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>197</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39">
+        <v>20</v>
+      </c>
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42" t="s">
+        <v>68</v>
+      </c>
+      <c r="D42">
+        <v>30</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43">
+        <v>23</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44">
+        <v>59</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45">
+        <v>3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>73</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47">
+        <v>26</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>74</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48">
+        <v>20</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49">
+        <v>3</v>
+      </c>
+      <c r="C49" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>78</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52">
+        <v>54</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>80</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>81</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>82</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>48</v>
+      </c>
+      <c r="D55">
+        <v>242</v>
+      </c>
+      <c r="E55" t="s">
+        <v>83</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>59</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>20</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>588</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>86</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>20</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>203</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>462</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>359</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>467</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>249</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>46</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>29</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>3</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>280</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>220</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>615</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>46</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>20</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>47</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>115</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>615</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>264</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>235</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>20</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>46</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>33</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>23</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>6</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-18)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -7,13 +7,14 @@
     <sheet sheetId="1" name="2026-09-15" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="2026-09-16" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="2026-09-17" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="2026-09-18" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1992" uniqueCount="156">
   <si>
     <t>이름</t>
   </si>
@@ -8352,6 +8353,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>1028</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>996</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>856</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>166</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>270</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>74</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>179</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>277</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>69</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>197</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39">
+        <v>20</v>
+      </c>
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42" t="s">
+        <v>68</v>
+      </c>
+      <c r="D42">
+        <v>30</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43">
+        <v>23</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44">
+        <v>59</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45">
+        <v>3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>73</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47">
+        <v>26</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>74</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48">
+        <v>20</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49">
+        <v>3</v>
+      </c>
+      <c r="C49" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>78</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52">
+        <v>54</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>80</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>81</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>82</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>83</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>350</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>59</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>20</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>856</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>86</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>20</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>439</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>515</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>657</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>700</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>352</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>46</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>29</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>3</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>363</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>523</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>933</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>46</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>20</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>47</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>115</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>645</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>352</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>273</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>30</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>46</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>33</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>23</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>6</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-19)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -8,13 +8,14 @@
     <sheet sheetId="2" name="2026-09-16" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="2026-09-17" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="2026-09-18" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="2026-09-19" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1992" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2490" uniqueCount="156">
   <si>
     <t>이름</t>
   </si>
@@ -10852,6 +10853,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>65</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>1311</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>1106</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>1096</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>269</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>273</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>74</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>179</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>277</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>79</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>197</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39">
+        <v>20</v>
+      </c>
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42" t="s">
+        <v>68</v>
+      </c>
+      <c r="D42">
+        <v>30</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43">
+        <v>23</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44">
+        <v>157</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45">
+        <v>3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>73</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47">
+        <v>26</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>74</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48">
+        <v>20</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49">
+        <v>3</v>
+      </c>
+      <c r="C49" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>78</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52">
+        <v>54</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>80</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>81</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>82</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>83</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>428</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>59</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>20</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>929</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>86</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>20</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>449</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>778</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>935</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>938</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>380</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>46</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>29</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>3</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>363</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>1019</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>1146</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>46</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>20</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>47</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>115</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>928</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>615</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>281</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>30</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>46</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>53</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>23</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>6</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-20)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -9,13 +9,14 @@
     <sheet sheetId="3" name="2026-09-17" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="2026-09-18" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="2026-09-19" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="2026-09-20" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2490" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="156">
   <si>
     <t>이름</t>
   </si>
@@ -13352,6 +13353,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>65</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>1639</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>1454</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>1399</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>544</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>276</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>127</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>179</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>490</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>79</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>197</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38">
+        <v>3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39">
+        <v>20</v>
+      </c>
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42" t="s">
+        <v>68</v>
+      </c>
+      <c r="D42">
+        <v>30</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43">
+        <v>23</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44">
+        <v>260</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>71</v>
+      </c>
+      <c r="B45">
+        <v>3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>73</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D47">
+        <v>26</v>
+      </c>
+      <c r="E47" t="s">
+        <v>8</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>74</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48">
+        <v>20</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49">
+        <v>3</v>
+      </c>
+      <c r="C49" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>78</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>64</v>
+      </c>
+      <c r="D52">
+        <v>64</v>
+      </c>
+      <c r="E52" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>80</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>81</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>82</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>48</v>
+      </c>
+      <c r="D55">
+        <v>466</v>
+      </c>
+      <c r="E55" t="s">
+        <v>83</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>59</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>33</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>20</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>1192</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>86</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>20</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>787</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>778</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>1053</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>1231</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>458</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>69</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>29</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>3</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>616</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>1182</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>1409</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>46</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>20</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>3</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>55</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>115</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>1276</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>1126</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>289</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>30</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>59</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>53</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>23</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>6</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-21)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="2026-09-18" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="2026-09-19" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="2026-09-20" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="2026-09-21" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3486" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -485,6 +486,9 @@
   <si>
     <t>황성욱</t>
   </si>
+  <si>
+    <t>김효준</t>
+  </si>
 </sst>
 </file>
 
@@ -15852,6 +15856,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>88</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>2007</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>2112</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>39</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>1742</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>692</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>299</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>147</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>472</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>1101</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>102</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>217</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>40</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>50</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>303</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>40</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>188</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>504</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>82</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>33</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>40</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>1590</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>86</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>51</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>807</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>798</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>1286</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>1251</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>486</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>92</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>52</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>51</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>839</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>1527</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>20</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>1800</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>69</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>40</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>3</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>75</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>125</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>1584</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>1231</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>424</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>50</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>79</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>73</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>311</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>6</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-22)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -11,13 +11,14 @@
     <sheet sheetId="5" name="2026-09-19" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="2026-09-20" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="2026-09-21" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="2026-09-22" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3486" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3988" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -18355,6 +18356,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>88</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>2468</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>2185</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>39</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>2213</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>920</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>355</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>157</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>472</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>1181</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>102</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>217</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>40</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>50</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>303</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>40</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>221</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>507</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>82</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>33</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>1958</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>61</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>965</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>801</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1389</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>1689</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>522</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>92</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>52</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>71</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>839</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>1948</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>20</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>2203</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>69</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>40</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>3</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>125</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>1910</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>1932</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>435</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>50</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>79</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>73</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>311</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-23)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -12,13 +12,14 @@
     <sheet sheetId="6" name="2026-09-20" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="2026-09-21" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="2026-09-22" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="2026-09-23" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3988" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4490" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -20875,6 +20876,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>91</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>72</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>2938</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>2636</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>72</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>2608</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1088</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>418</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>157</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>910</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>1514</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>125</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>217</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>40</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>50</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>303</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>40</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>234</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>545</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>82</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>33</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>2721</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>64</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>978</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>804</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1502</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>1782</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>700</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>92</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>55</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>71</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>942</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>2394</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>30</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>2731</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>69</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>40</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>6</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>128</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>1920</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>2022</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>553</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>50</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>79</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>83</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>311</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-24)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -13,13 +13,14 @@
     <sheet sheetId="7" name="2026-09-21" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="2026-09-22" state="visible" r:id="rId11"/>
     <sheet sheetId="9" name="2026-09-23" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="2026-09-24" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4490" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4992" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -3367,6 +3368,2525 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>94</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>125</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>3356</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>3151</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>72</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>3104</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1199</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>501</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>157</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>910</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>1957</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>125</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>217</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>50</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>50</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>303</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>40</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>234</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>646</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>82</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>33</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>2807</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>64</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>981</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>804</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1505</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>1830</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>700</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>92</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>55</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>71</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1015</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>2824</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>30</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>3229</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>69</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>40</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>6</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>128</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2143</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>2430</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>561</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>50</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>79</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>83</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>311</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F124"/>
@@ -23395,6 +25915,6 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-25)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -14,13 +14,14 @@
     <sheet sheetId="8" name="2026-09-22" state="visible" r:id="rId11"/>
     <sheet sheetId="9" name="2026-09-23" state="visible" r:id="rId12"/>
     <sheet sheetId="10" name="2026-09-24" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="2026-09-25" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4992" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5494" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -5883,6 +5884,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>94</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>125</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>3904</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>3724</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>3629</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1254</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>501</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>157</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>910</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>2155</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>125</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>217</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>50</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>50</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>311</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>40</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>237</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>649</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>82</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>33</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>3220</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>64</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>984</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1107</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1505</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>1830</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>700</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>92</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>55</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>71</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1015</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>3202</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>30</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>3740</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>69</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>40</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>6</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>138</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2153</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>2843</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>564</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>79</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>83</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>311</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-26)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -15,13 +15,14 @@
     <sheet sheetId="9" name="2026-09-23" state="visible" r:id="rId12"/>
     <sheet sheetId="10" name="2026-09-24" state="visible" r:id="rId13"/>
     <sheet sheetId="11" name="2026-09-25" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="2026-09-26" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5494" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5996" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -8403,6 +8404,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>97</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>125</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>4367</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>4152</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>4012</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1350</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>514</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>157</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>1213</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>2298</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>125</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>217</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>50</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>50</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>311</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>40</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>237</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>705</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>82</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>36</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>3543</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>64</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1107</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1140</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1613</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>1830</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>718</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>92</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>55</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>71</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1218</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>3788</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>30</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>4030</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>69</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>40</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>6</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>148</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2163</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>3226</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>842</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>79</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>83</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>311</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-27)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -16,13 +16,14 @@
     <sheet sheetId="10" name="2026-09-24" state="visible" r:id="rId13"/>
     <sheet sheetId="11" name="2026-09-25" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="2026-09-26" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="2026-09-27" state="visible" r:id="rId16"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5996" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6498" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -10923,6 +10924,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>97</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>125</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>4850</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>4515</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>69</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>81</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>4410</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1380</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>517</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>157</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>1416</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>2519</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>125</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>217</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>50</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>50</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>411</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>40</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>84</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>237</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>713</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>82</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>36</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>3906</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>64</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1107</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1140</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1613</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>1833</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>726</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>135</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>58</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>94</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1301</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>3828</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>30</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>4423</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>69</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>40</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>6</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>148</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2506</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>3254</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>850</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>82</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>83</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>311</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-28)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -17,13 +17,14 @@
     <sheet sheetId="11" name="2026-09-25" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="2026-09-26" state="visible" r:id="rId15"/>
     <sheet sheetId="13" name="2026-09-27" state="visible" r:id="rId16"/>
+    <sheet sheetId="14" name="2026-09-28" state="visible" r:id="rId17"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6498" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7000" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -13443,6 +13444,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>148</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>5348</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>5018</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>92</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>104</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>4898</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1441</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>543</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>177</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>1849</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>2884</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>178</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>237</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>60</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>70</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>70</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>439</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>260</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>741</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>105</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>56</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>4296</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>122</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1275</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1258</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1671</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2251</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1149</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>168</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>78</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>124</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1379</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>4014</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>53</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>4846</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>92</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>60</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>29</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>20</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>168</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2546</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>3284</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>870</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>102</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>103</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>463</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>20</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>419</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-29)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -18,13 +18,14 @@
     <sheet sheetId="12" name="2026-09-26" state="visible" r:id="rId15"/>
     <sheet sheetId="13" name="2026-09-27" state="visible" r:id="rId16"/>
     <sheet sheetId="14" name="2026-09-28" state="visible" r:id="rId17"/>
+    <sheet sheetId="15" name="2026-09-29" state="visible" r:id="rId18"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7000" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7502" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -15963,6 +15964,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>148</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>5866</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>5421</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>105</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>114</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>5301</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1504</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>543</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>177</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>2252</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>3107</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>178</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>237</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>60</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>70</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>70</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>449</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>260</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>744</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>105</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>79</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>4692</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>86</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>122</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1275</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1258</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1671</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2251</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1292</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>168</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>91</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>137</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1379</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>4454</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>53</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>5159</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>92</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>60</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>29</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>20</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>171</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2546</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>3707</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1246</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>102</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>103</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>1284</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>20</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>419</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-09-30)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -19,13 +19,14 @@
     <sheet sheetId="13" name="2026-09-27" state="visible" r:id="rId16"/>
     <sheet sheetId="14" name="2026-09-28" state="visible" r:id="rId17"/>
     <sheet sheetId="15" name="2026-09-29" state="visible" r:id="rId18"/>
+    <sheet sheetId="16" name="2026-09-30" state="visible" r:id="rId19"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7502" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8000" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -18483,6 +18484,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>176</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>6459</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>5997</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>105</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>114</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>5329</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1574</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>543</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>177</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>2252</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>3510</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>178</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>237</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>60</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>70</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>70</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>449</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>260</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>787</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>115</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>79</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>40</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>5075</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>96</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>122</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>1275</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>1258</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>1774</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>2251</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>1375</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>178</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>91</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>137</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>1452</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>4787</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>53</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>5882</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>92</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>60</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>29</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>3</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>20</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>85</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>171</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>2546</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>3950</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>1246</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>60</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>102</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>103</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>1304</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>20</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>419</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>6</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-01)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -20,13 +20,14 @@
     <sheet sheetId="14" name="2026-09-28" state="visible" r:id="rId17"/>
     <sheet sheetId="15" name="2026-09-29" state="visible" r:id="rId18"/>
     <sheet sheetId="16" name="2026-09-30" state="visible" r:id="rId19"/>
+    <sheet sheetId="17" name="2026-10-01" state="visible" r:id="rId20"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8000" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8502" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -20983,6 +20984,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>176</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>7082</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>6552</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>105</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>114</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>5782</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1607</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>556</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>177</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>2675</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>3540</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>231</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>237</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>60</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>70</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>70</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>449</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>260</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>800</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>115</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>79</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>5478</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>96</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>122</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1398</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1258</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1774</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2261</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1441</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>178</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>91</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>147</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1462</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>5230</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>63</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>6565</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>92</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>60</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>29</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>20</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>181</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2546</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4013</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1344</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>102</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>103</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>1677</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>20</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>429</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-02)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -21,13 +21,14 @@
     <sheet sheetId="15" name="2026-09-29" state="visible" r:id="rId18"/>
     <sheet sheetId="16" name="2026-09-30" state="visible" r:id="rId19"/>
     <sheet sheetId="17" name="2026-10-01" state="visible" r:id="rId20"/>
+    <sheet sheetId="18" name="2026-10-02" state="visible" r:id="rId21"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8502" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9004" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -23503,6 +23504,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>204</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>8128</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>7218</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>115</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>167</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>5802</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1698</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>559</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>177</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>3083</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>3993</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>234</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>237</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>60</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>70</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>70</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>449</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>270</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1353</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>115</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>79</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>5871</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>96</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>130</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1491</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1258</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1774</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2269</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1486</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>178</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>91</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>147</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1595</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>5626</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>63</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>7336</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>92</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>60</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>29</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>20</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>85</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>184</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2546</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4056</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1375</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>102</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>103</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>1677</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>23</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>429</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-03)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -22,13 +22,14 @@
     <sheet sheetId="16" name="2026-09-30" state="visible" r:id="rId19"/>
     <sheet sheetId="17" name="2026-10-01" state="visible" r:id="rId20"/>
     <sheet sheetId="18" name="2026-10-02" state="visible" r:id="rId21"/>
+    <sheet sheetId="19" name="2026-10-03" state="visible" r:id="rId22"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9004" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9506" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -26023,6 +26024,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>123</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>204</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>8686</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>7498</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>125</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>167</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>6260</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1733</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>562</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>177</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>3546</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>4406</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>234</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>237</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>60</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>70</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>70</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>480</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>280</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1386</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>125</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>79</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>40</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>6389</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>96</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>133</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>26</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1491</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1258</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1774</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2269</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1504</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>178</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>91</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>147</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1595</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>5966</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>83</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>7826</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>92</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>60</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>29</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>20</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>98</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>184</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>2556</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4099</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1378</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>60</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>102</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>123</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>1677</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>23</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>429</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>6</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-04)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -23,13 +23,14 @@
     <sheet sheetId="17" name="2026-10-01" state="visible" r:id="rId20"/>
     <sheet sheetId="18" name="2026-10-02" state="visible" r:id="rId21"/>
     <sheet sheetId="19" name="2026-10-03" state="visible" r:id="rId22"/>
+    <sheet sheetId="20" name="2026-10-04" state="visible" r:id="rId23"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9506" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10004" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -28543,7 +28544,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -31043,6 +31044,2505 @@
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>123</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>204</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>8714</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>8031</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>33</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>135</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>167</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>6633</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1751</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>562</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>177</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>4004</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>4829</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>60</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>257</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>237</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>43</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>60</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>70</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>70</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>43</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>490</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>46</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>60</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>107</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>280</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1404</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>125</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>79</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>40</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>6842</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>96</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>133</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>26</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>1491</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>1258</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>1872</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>2269</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>1572</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>178</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>91</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>147</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>1671</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>6292</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>83</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>8272</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>92</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>60</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>29</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>86</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>20</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>101</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>184</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>2556</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>4542</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>1388</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>60</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>102</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>123</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>1680</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>23</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>429</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>6</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-05)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -24,13 +24,14 @@
     <sheet sheetId="18" name="2026-10-02" state="visible" r:id="rId21"/>
     <sheet sheetId="19" name="2026-10-03" state="visible" r:id="rId22"/>
     <sheet sheetId="20" name="2026-10-04" state="visible" r:id="rId23"/>
+    <sheet sheetId="21" name="2026-10-05" state="visible" r:id="rId24"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10004" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10506" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -33542,6 +33543,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>376</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>477</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>9634</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>9018</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>435</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>627</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7193</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>2059</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>815</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>522</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>4487</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>5747</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>547</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>330</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>310</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>433</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>360</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>370</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>313</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1036</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>280</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>477</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>650</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>2077</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>375</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>529</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>340</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>7585</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>508</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>426</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>290</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3474</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1608</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>2172</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2589</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1950</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>431</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>330</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>514</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>470</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>1961</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>6820</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>9219</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>392</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>510</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>429</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>336</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>637</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3056</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4910</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>360</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1644</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>483</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>472</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>623</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>1990</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>313</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1237</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>259</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-06)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -25,13 +25,14 @@
     <sheet sheetId="19" name="2026-10-03" state="visible" r:id="rId22"/>
     <sheet sheetId="20" name="2026-10-04" state="visible" r:id="rId23"/>
     <sheet sheetId="21" name="2026-10-05" state="visible" r:id="rId24"/>
+    <sheet sheetId="22" name="2026-10-06" state="visible" r:id="rId25"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10506" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11004" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -36062,6 +36063,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>379</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>477</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>10400</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>9018</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>438</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>627</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7211</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>2112</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>815</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>532</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>4487</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>6150</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>550</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>330</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>310</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>360</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>370</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>313</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1036</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>280</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>477</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>653</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>2618</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>280</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>375</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>529</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>370</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>340</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>7868</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>250</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>546</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>290</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>370</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>508</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>426</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>290</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>400</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>250</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>370</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>3477</v>
+      </c>
+      <c r="E73" t="s">
+        <v>83</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>400</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>290</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>1608</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>2182</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>2677</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>280</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>2043</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>370</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>310</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>464</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>330</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>250</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>350</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>517</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>490</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>250</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>370</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>2327</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>7000</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>310</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>483</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>9632</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>392</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>510</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>429</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>280</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>336</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>422</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>471</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>637</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>370</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>3056</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>4948</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>370</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>290</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>360</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>1677</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>483</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>482</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>280</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>250</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>623</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>1990</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>323</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>1237</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>250</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>370</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>262</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-07)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -26,13 +26,14 @@
     <sheet sheetId="20" name="2026-10-04" state="visible" r:id="rId23"/>
     <sheet sheetId="21" name="2026-10-05" state="visible" r:id="rId24"/>
     <sheet sheetId="22" name="2026-10-06" state="visible" r:id="rId25"/>
+    <sheet sheetId="23" name="2026-10-07" state="visible" r:id="rId26"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11004" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11506" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -38562,6 +38563,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>379</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>10860</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>9411</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>438</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>627</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7534</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1855</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>815</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>532</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>4507</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>6543</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>550</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>330</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>310</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>360</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>370</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>313</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1039</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>280</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>477</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>653</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>2623</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>375</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>529</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>340</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>8231</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>508</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>426</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>290</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3480</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1608</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>2210</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2970</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>2043</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>464</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>330</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>517</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>500</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2347</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>7383</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>10265</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>392</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>510</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>429</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>336</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>637</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3056</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>5011</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>360</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1755</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>483</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>482</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>623</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2000</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>326</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1237</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-08)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -27,13 +27,14 @@
     <sheet sheetId="21" name="2026-10-05" state="visible" r:id="rId24"/>
     <sheet sheetId="22" name="2026-10-06" state="visible" r:id="rId25"/>
     <sheet sheetId="23" name="2026-10-07" state="visible" r:id="rId26"/>
+    <sheet sheetId="24" name="2026-10-08" state="visible" r:id="rId27"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11506" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12008" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -41082,6 +41083,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>382</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>11516</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>9809</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>441</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>627</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7534</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1648</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>618</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>532</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>4890</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>6449</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>563</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>330</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>310</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>360</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>370</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>313</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1122</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>280</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>477</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>653</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>2691</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>375</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>529</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>340</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>8676</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>508</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>426</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>290</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3483</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1608</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>2238</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2980</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>2053</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>464</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>330</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>527</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>500</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2527</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>8059</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>10768</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>392</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>510</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>429</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>336</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>637</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3056</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4904</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>360</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1538</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>483</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>482</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>623</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2000</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>326</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1237</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-09)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -28,13 +28,14 @@
     <sheet sheetId="22" name="2026-10-06" state="visible" r:id="rId25"/>
     <sheet sheetId="23" name="2026-10-07" state="visible" r:id="rId26"/>
     <sheet sheetId="24" name="2026-10-08" state="visible" r:id="rId27"/>
+    <sheet sheetId="25" name="2026-10-09" state="visible" r:id="rId28"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12008" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12510" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -43602,6 +43603,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>382</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>523</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>12076</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>9822</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>441</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>627</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7534</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1571</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>618</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>532</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5103</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>6362</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>563</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>330</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>310</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>360</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>370</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>323</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1510</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>280</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>477</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>653</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>2439</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>375</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>529</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>340</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>9122</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>508</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>426</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>290</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3546</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1608</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>2164</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>3103</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>2053</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>464</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>330</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>530</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>500</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2527</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>8144</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>11181</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>392</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>510</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>429</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>336</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>637</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3056</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4990</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>360</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1331</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>483</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>482</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>623</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2000</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>326</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1237</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-10)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -29,13 +29,14 @@
     <sheet sheetId="23" name="2026-10-07" state="visible" r:id="rId26"/>
     <sheet sheetId="24" name="2026-10-08" state="visible" r:id="rId27"/>
     <sheet sheetId="25" name="2026-10-09" state="visible" r:id="rId28"/>
+    <sheet sheetId="26" name="2026-10-10" state="visible" r:id="rId29"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12510" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13012" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -46122,6 +46123,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>382</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>546</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>12769</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>10222</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>441</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>660</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7534</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1359</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>661</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>532</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5103</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>6300</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>566</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>330</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>310</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>360</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>370</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>323</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1510</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>280</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>477</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>653</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>2147</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>385</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>545</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>340</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>9680</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>508</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>426</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>290</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3662</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1608</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>2104</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2906</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1866</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>464</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>330</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>533</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>500</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2527</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>8587</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>11181</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>392</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>510</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>429</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>336</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>637</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3099</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>5090</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>360</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1239</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>483</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>482</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>623</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2000</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>326</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1237</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-11)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -30,13 +30,14 @@
     <sheet sheetId="24" name="2026-10-08" state="visible" r:id="rId27"/>
     <sheet sheetId="25" name="2026-10-09" state="visible" r:id="rId28"/>
     <sheet sheetId="26" name="2026-10-10" state="visible" r:id="rId29"/>
+    <sheet sheetId="27" name="2026-10-11" state="visible" r:id="rId30"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13012" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13514" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -48642,6 +48643,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>382</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>546</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>13362</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>10680</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>441</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>663</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7982</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1382</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>664</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>532</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5103</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>6820</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>566</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>330</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>310</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>360</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>370</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>323</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1538</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>280</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>477</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>653</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1852</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>385</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>340</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>10125</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>508</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>426</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>290</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3362</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1856</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1977</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2979</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1624</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>464</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>333</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>536</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>500</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>9050</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>11774</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>392</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>510</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>432</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>99</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>637</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3099</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>5118</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>360</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1139</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>493</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>482</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>623</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2000</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>326</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1237</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-12)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -31,13 +31,14 @@
     <sheet sheetId="25" name="2026-10-09" state="visible" r:id="rId28"/>
     <sheet sheetId="26" name="2026-10-10" state="visible" r:id="rId29"/>
     <sheet sheetId="27" name="2026-10-11" state="visible" r:id="rId30"/>
+    <sheet sheetId="28" name="2026-10-12" state="visible" r:id="rId31"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13514" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14016" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -51162,6 +51163,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>385</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>564</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>14323</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>10783</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>444</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>7965</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1382</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>667</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>552</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5153</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>7193</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>569</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1596</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>480</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>686</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1678</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>408</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>10628</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1621</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>459</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>343</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3405</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1844</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1980</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>3002</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1390</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>487</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>536</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>550</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>9846</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>12507</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>415</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>432</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>109</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>765</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3179</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>5016</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>393</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1112</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>503</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>505</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>673</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2020</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>326</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1490</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-13)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -32,13 +32,14 @@
     <sheet sheetId="26" name="2026-10-10" state="visible" r:id="rId29"/>
     <sheet sheetId="27" name="2026-10-11" state="visible" r:id="rId30"/>
     <sheet sheetId="28" name="2026-10-12" state="visible" r:id="rId31"/>
+    <sheet sheetId="29" name="2026-10-13" state="visible" r:id="rId32"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14016" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14518" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -53682,6 +53683,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>385</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>592</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>14866</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>11361</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>444</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>8478</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>1125</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>670</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>552</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5163</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>7556</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>569</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1599</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>480</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>686</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1478</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>408</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>11149</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>546</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1532</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>459</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3438</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1857</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1806</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>3002</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1400</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>487</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>539</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>550</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>9906</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>12905</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>415</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>432</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>2</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>813</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3209</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4922</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>393</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>1045</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>503</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>508</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>703</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2030</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>326</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1490</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-14)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -33,13 +33,14 @@
     <sheet sheetId="27" name="2026-10-11" state="visible" r:id="rId30"/>
     <sheet sheetId="28" name="2026-10-12" state="visible" r:id="rId31"/>
     <sheet sheetId="29" name="2026-10-13" state="visible" r:id="rId32"/>
+    <sheet sheetId="30" name="2026-10-14" state="visible" r:id="rId33"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14518" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15020" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -56202,7 +56203,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -58702,6 +58703,2525 @@
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>388</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>602</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>14986</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>11854</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>454</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>8666</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>891</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>683</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>552</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5163</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>7914</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>569</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1602</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>350</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>480</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>686</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1484</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>408</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>11789</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>566</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1595</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>459</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3501</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1857</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1579</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2785</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1183</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>539</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>550</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>9879</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>13733</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>415</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>432</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>15</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>956</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3209</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>5002</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>961</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>503</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>508</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>713</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2030</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>329</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1490</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-15)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -34,13 +34,14 @@
     <sheet sheetId="28" name="2026-10-12" state="visible" r:id="rId31"/>
     <sheet sheetId="29" name="2026-10-13" state="visible" r:id="rId32"/>
     <sheet sheetId="30" name="2026-10-14" state="visible" r:id="rId33"/>
+    <sheet sheetId="31" name="2026-10-15" state="visible" r:id="rId34"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15020" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15522" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -61221,6 +61222,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>391</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>625</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>15472</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>12367</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>474</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>8669</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>631</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>721</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>552</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5163</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>7627</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>569</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>310</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1602</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>360</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>483</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>686</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1484</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>408</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>12262</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>566</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1610</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>459</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3504</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1860</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1579</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2588</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1186</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>539</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>10352</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>14386</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>415</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>438</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>959</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3209</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>5265</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>949</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>503</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>508</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>713</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2030</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>339</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1490</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-16)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -35,13 +35,14 @@
     <sheet sheetId="29" name="2026-10-13" state="visible" r:id="rId32"/>
     <sheet sheetId="30" name="2026-10-14" state="visible" r:id="rId33"/>
     <sheet sheetId="31" name="2026-10-15" state="visible" r:id="rId34"/>
+    <sheet sheetId="32" name="2026-10-16" state="visible" r:id="rId35"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15522" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16024" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -63741,6 +63742,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>391</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>625</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>15832</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>12853</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>507</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>8762</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>464</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>779</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>552</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5173</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>7935</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>569</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1602</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>360</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>483</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>686</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1487</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>408</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>12678</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>566</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1653</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>459</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3507</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1973</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1662</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2588</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1189</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>539</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>10585</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>14386</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>415</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>438</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>972</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3209</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>5131</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>859</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>503</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>508</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>713</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2040</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>342</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1490</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-17)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -36,13 +36,14 @@
     <sheet sheetId="30" name="2026-10-14" state="visible" r:id="rId33"/>
     <sheet sheetId="31" name="2026-10-15" state="visible" r:id="rId34"/>
     <sheet sheetId="32" name="2026-10-16" state="visible" r:id="rId35"/>
+    <sheet sheetId="33" name="2026-10-17" state="visible" r:id="rId36"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16024" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16526" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -66261,6 +66262,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>391</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>653</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>16485</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>13253</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>507</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>8772</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>257</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>792</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>552</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5173</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>8258</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>569</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>333</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1602</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>360</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>483</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>686</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1295</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>408</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>12726</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>566</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1691</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>459</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3507</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>2041</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1572</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2588</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1199</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>539</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>10988</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>14944</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>415</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>438</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>1085</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3219</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4974</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>895</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>503</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>508</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>713</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2040</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>342</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1490</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-18)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -37,13 +37,14 @@
     <sheet sheetId="31" name="2026-10-15" state="visible" r:id="rId34"/>
     <sheet sheetId="32" name="2026-10-16" state="visible" r:id="rId35"/>
     <sheet sheetId="33" name="2026-10-17" state="visible" r:id="rId36"/>
+    <sheet sheetId="34" name="2026-10-18" state="visible" r:id="rId37"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16526" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17028" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -68781,6 +68782,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>391</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>653</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>16858</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>13786</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>507</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>9000</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>315</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>795</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>558</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5173</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>8681</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>569</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>637</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>443</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1602</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>360</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>483</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>692</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1295</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>408</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>13159</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>566</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1729</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>459</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3440</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>2054</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1575</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2588</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>1022</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>542</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>11211</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>483</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>14944</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>415</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>1834</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>471</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>1153</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3219</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4927</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>623</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>503</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>508</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>713</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2040</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>342</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1490</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>250</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-19)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -38,13 +38,14 @@
     <sheet sheetId="32" name="2026-10-16" state="visible" r:id="rId35"/>
     <sheet sheetId="33" name="2026-10-17" state="visible" r:id="rId36"/>
     <sheet sheetId="34" name="2026-10-18" state="visible" r:id="rId37"/>
+    <sheet sheetId="35" name="2026-10-19" state="visible" r:id="rId38"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17028" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17526" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -71301,6 +71302,2505 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>394</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>656</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>17486</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>14332</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>510</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>9303</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>326</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>798</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>608</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5173</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>9214</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>572</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>730</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>446</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1602</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>363</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>486</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>692</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1208</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57">
+        <v>280</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>86</v>
+      </c>
+      <c r="D58">
+        <v>418</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>87</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>48</v>
+      </c>
+      <c r="D59">
+        <v>658</v>
+      </c>
+      <c r="E59" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60">
+        <v>370</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>89</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61">
+        <v>360</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62">
+        <v>13769</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63">
+        <v>250</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>92</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64">
+        <v>566</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>290</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>94</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66">
+        <v>370</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>1792</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D68">
+        <v>692</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>97</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>383</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70">
+        <v>400</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>99</v>
+      </c>
+      <c r="B71">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71">
+        <v>250</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>100</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72">
+        <v>370</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>3643</v>
+      </c>
+      <c r="E73" t="s">
+        <v>83</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>31</v>
+      </c>
+      <c r="D74">
+        <v>400</v>
+      </c>
+      <c r="E74" t="s">
+        <v>14</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>66</v>
+      </c>
+      <c r="D75">
+        <v>290</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76">
+        <v>2057</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77">
+        <v>1575</v>
+      </c>
+      <c r="E77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78">
+        <v>2</v>
+      </c>
+      <c r="C78" t="s">
+        <v>107</v>
+      </c>
+      <c r="D78">
+        <v>2591</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79">
+        <v>280</v>
+      </c>
+      <c r="E79" t="s">
+        <v>14</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>109</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80">
+        <v>825</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81">
+        <v>370</v>
+      </c>
+      <c r="E81" t="s">
+        <v>14</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82">
+        <v>2</v>
+      </c>
+      <c r="C82" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>40</v>
+      </c>
+      <c r="D83">
+        <v>310</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>86</v>
+      </c>
+      <c r="D84">
+        <v>570</v>
+      </c>
+      <c r="E84" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>114</v>
+      </c>
+      <c r="B85">
+        <v>2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>40</v>
+      </c>
+      <c r="D85">
+        <v>363</v>
+      </c>
+      <c r="E85" t="s">
+        <v>14</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>250</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88">
+        <v>2</v>
+      </c>
+      <c r="C88" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88">
+        <v>350</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+      <c r="C89" t="s">
+        <v>31</v>
+      </c>
+      <c r="D89">
+        <v>542</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>68</v>
+      </c>
+      <c r="D90">
+        <v>560</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>250</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92">
+        <v>370</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>2780</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95">
+        <v>12167</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>40</v>
+      </c>
+      <c r="D96">
+        <v>310</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>43</v>
+      </c>
+      <c r="D97">
+        <v>696</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>40</v>
+      </c>
+      <c r="D98">
+        <v>15147</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>425</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100">
+        <v>560</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>43</v>
+      </c>
+      <c r="D101">
+        <v>435</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>131</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>280</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>132</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>1834</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>133</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104">
+        <v>422</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>134</v>
+      </c>
+      <c r="B105">
+        <v>1</v>
+      </c>
+      <c r="C105" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105">
+        <v>474</v>
+      </c>
+      <c r="E105" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>136</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106">
+        <v>1206</v>
+      </c>
+      <c r="E106" t="s">
+        <v>14</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>24</v>
+      </c>
+      <c r="D107">
+        <v>370</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>138</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108">
+        <v>3762</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>139</v>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="s">
+        <v>26</v>
+      </c>
+      <c r="D109">
+        <v>4937</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>140</v>
+      </c>
+      <c r="B110">
+        <v>1</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110">
+        <v>370</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>141</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111">
+        <v>290</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>142</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>40</v>
+      </c>
+      <c r="D112">
+        <v>403</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>143</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113">
+        <v>766</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>144</v>
+      </c>
+      <c r="B114">
+        <v>1</v>
+      </c>
+      <c r="C114" t="s">
+        <v>43</v>
+      </c>
+      <c r="D114">
+        <v>513</v>
+      </c>
+      <c r="E114" t="s">
+        <v>14</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>145</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>16</v>
+      </c>
+      <c r="D115">
+        <v>511</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>146</v>
+      </c>
+      <c r="B116">
+        <v>3</v>
+      </c>
+      <c r="C116" t="s">
+        <v>13</v>
+      </c>
+      <c r="D116">
+        <v>280</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>147</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>148</v>
+      </c>
+      <c r="D117">
+        <v>250</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>149</v>
+      </c>
+      <c r="B118">
+        <v>1</v>
+      </c>
+      <c r="C118" t="s">
+        <v>48</v>
+      </c>
+      <c r="D118">
+        <v>783</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>150</v>
+      </c>
+      <c r="B119">
+        <v>3</v>
+      </c>
+      <c r="C119" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119">
+        <v>2040</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>151</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>20</v>
+      </c>
+      <c r="D120">
+        <v>342</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>152</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>31</v>
+      </c>
+      <c r="D121">
+        <v>1253</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>153</v>
+      </c>
+      <c r="B122">
+        <v>3</v>
+      </c>
+      <c r="C122" t="s">
+        <v>26</v>
+      </c>
+      <c r="D122">
+        <v>1163</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>154</v>
+      </c>
+      <c r="B123">
+        <v>1</v>
+      </c>
+      <c r="C123" t="s">
+        <v>24</v>
+      </c>
+      <c r="D123">
+        <v>370</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124" t="s">
+        <v>7</v>
+      </c>
+      <c r="D124">
+        <v>262</v>
+      </c>
+      <c r="E124" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-20)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -39,13 +39,14 @@
     <sheet sheetId="33" name="2026-10-17" state="visible" r:id="rId36"/>
     <sheet sheetId="34" name="2026-10-18" state="visible" r:id="rId37"/>
     <sheet sheetId="35" name="2026-10-19" state="visible" r:id="rId38"/>
+    <sheet sheetId="36" name="2026-10-20" state="visible" r:id="rId39"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17526" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18028" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -73801,6 +73802,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>394</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>666</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>17969</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>15710</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>520</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>9521</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>66</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>821</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>611</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5593</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>9847</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>572</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>730</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>446</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>1602</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>363</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>486</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>692</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1211</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>431</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>658</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>14455</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>566</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1845</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>692</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3646</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1980</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1600</v>
+      </c>
+      <c r="E78" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2591</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>825</v>
+      </c>
+      <c r="E81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>542</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>12230</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>696</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>16110</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>445</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>2152</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>474</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>1124</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3765</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4700</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>779</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>513</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>511</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>803</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2040</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>1195</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1253</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>1163</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-21)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -40,13 +40,14 @@
     <sheet sheetId="34" name="2026-10-18" state="visible" r:id="rId37"/>
     <sheet sheetId="35" name="2026-10-19" state="visible" r:id="rId38"/>
     <sheet sheetId="36" name="2026-10-20" state="visible" r:id="rId39"/>
+    <sheet sheetId="37" name="2026-10-21" state="visible" r:id="rId40"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18028" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18530" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -76321,6 +76322,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>394</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>689</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>18399</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>15723</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>520</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>839</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>9521</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>9</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>824</v>
+      </c>
+      <c r="E20" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>611</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5666</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>10490</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>575</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>730</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>446</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>2440</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>296</v>
+      </c>
+      <c r="E48" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>363</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>486</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>692</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1211</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>283</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59">
+        <v>431</v>
+      </c>
+      <c r="E59" t="s">
+        <v>8</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>668</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>15068</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>576</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1878</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>692</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>3649</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1990</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1378</v>
+      </c>
+      <c r="E78" t="s">
+        <v>83</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>107</v>
+      </c>
+      <c r="D79">
+        <v>2591</v>
+      </c>
+      <c r="E79" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>678</v>
+      </c>
+      <c r="E81" t="s">
+        <v>83</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>86</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>542</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>13323</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>310</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>696</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>16816</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>455</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>2435</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>474</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>1137</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3765</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4606</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>527</v>
+      </c>
+      <c r="E114" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>513</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>511</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>803</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2040</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>1195</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1253</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>1163</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>83</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-22)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -41,13 +41,14 @@
     <sheet sheetId="35" name="2026-10-19" state="visible" r:id="rId38"/>
     <sheet sheetId="36" name="2026-10-20" state="visible" r:id="rId39"/>
     <sheet sheetId="37" name="2026-10-21" state="visible" r:id="rId40"/>
+    <sheet sheetId="38" name="2026-10-22" state="visible" r:id="rId41"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18530" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19032" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -78841,6 +78842,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>394</v>
+      </c>
+      <c r="E2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>717</v>
+      </c>
+      <c r="E3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>19072</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>17011</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>520</v>
+      </c>
+      <c r="E8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>862</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>9551</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>85</v>
+      </c>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>350</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>727</v>
+      </c>
+      <c r="E20" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>611</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>5666</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>11103</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>578</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>730</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>83</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>446</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>83</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>450</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>2440</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>299</v>
+      </c>
+      <c r="E48" t="s">
+        <v>83</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>51</v>
+      </c>
+      <c r="D49">
+        <v>363</v>
+      </c>
+      <c r="E49" t="s">
+        <v>83</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>486</v>
+      </c>
+      <c r="E53" t="s">
+        <v>83</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>692</v>
+      </c>
+      <c r="E54" t="s">
+        <v>83</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57">
+        <v>1211</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>2623</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>22</v>
+      </c>
+      <c r="D59">
+        <v>431</v>
+      </c>
+      <c r="E59" t="s">
+        <v>83</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>668</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>15738</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>606</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>1991</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>692</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>2342</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>2010</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1161</v>
+      </c>
+      <c r="E78" t="s">
+        <v>83</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>51</v>
+      </c>
+      <c r="D79">
+        <v>2611</v>
+      </c>
+      <c r="E79" t="s">
+        <v>83</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>729</v>
+      </c>
+      <c r="E81" t="s">
+        <v>83</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>22</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>83</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>545</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>13388</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>340</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>696</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>17446</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>465</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>2723</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>474</v>
+      </c>
+      <c r="E106" t="s">
+        <v>83</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>1240</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3765</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4681</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>340</v>
+      </c>
+      <c r="E114" t="s">
+        <v>83</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>513</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>511</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>803</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2040</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>1195</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1253</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>1203</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>83</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-23)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -42,13 +42,14 @@
     <sheet sheetId="36" name="2026-10-20" state="visible" r:id="rId39"/>
     <sheet sheetId="37" name="2026-10-21" state="visible" r:id="rId40"/>
     <sheet sheetId="38" name="2026-10-22" state="visible" r:id="rId41"/>
+    <sheet sheetId="39" name="2026-10-23" state="visible" r:id="rId42"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19032" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19534" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -81361,6 +81362,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>394</v>
+      </c>
+      <c r="E2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>745</v>
+      </c>
+      <c r="E3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>19635</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>17051</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>520</v>
+      </c>
+      <c r="E8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>892</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>9999</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>55</v>
+      </c>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>360</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>640</v>
+      </c>
+      <c r="E20" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>611</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>7112</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>11606</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>578</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>730</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>83</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>446</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>83</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>460</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>2440</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>299</v>
+      </c>
+      <c r="E48" t="s">
+        <v>83</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>51</v>
+      </c>
+      <c r="D49">
+        <v>366</v>
+      </c>
+      <c r="E49" t="s">
+        <v>83</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>486</v>
+      </c>
+      <c r="E53" t="s">
+        <v>83</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>692</v>
+      </c>
+      <c r="E54" t="s">
+        <v>83</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1214</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>2643</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>22</v>
+      </c>
+      <c r="D59">
+        <v>431</v>
+      </c>
+      <c r="E59" t="s">
+        <v>83</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>668</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>16344</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>606</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>2034</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>692</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>2102</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>2031</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1164</v>
+      </c>
+      <c r="E78" t="s">
+        <v>83</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>51</v>
+      </c>
+      <c r="D79">
+        <v>2334</v>
+      </c>
+      <c r="E79" t="s">
+        <v>83</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>437</v>
+      </c>
+      <c r="E81" t="s">
+        <v>83</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>22</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>83</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>350</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>545</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>13831</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>350</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>696</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>18119</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>475</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3001</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>474</v>
+      </c>
+      <c r="E106" t="s">
+        <v>83</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>1240</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3765</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4744</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>348</v>
+      </c>
+      <c r="E114" t="s">
+        <v>83</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>513</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>511</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>3751</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2050</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>1798</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1253</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>1213</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>83</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-24)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -43,13 +43,14 @@
     <sheet sheetId="37" name="2026-10-21" state="visible" r:id="rId40"/>
     <sheet sheetId="38" name="2026-10-22" state="visible" r:id="rId41"/>
     <sheet sheetId="39" name="2026-10-23" state="visible" r:id="rId42"/>
+    <sheet sheetId="40" name="2026-10-24" state="visible" r:id="rId43"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19534" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20036" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -83881,7 +83882,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -86381,6 +86382,2525 @@
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>394</v>
+      </c>
+      <c r="E2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>745</v>
+      </c>
+      <c r="E3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>20268</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>18317</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>520</v>
+      </c>
+      <c r="E8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>350</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>892</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>10362</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>138</v>
+      </c>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>360</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>640</v>
+      </c>
+      <c r="E20" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>614</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25">
+        <v>290</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>7112</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27">
+        <v>12289</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>310</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29">
+        <v>588</v>
+      </c>
+      <c r="E29" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30">
+        <v>350</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31">
+        <v>730</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>250</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>156</v>
+      </c>
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>343</v>
+      </c>
+      <c r="E33" t="s">
+        <v>83</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34">
+        <v>330</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>370</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36">
+        <v>446</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>370</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39">
+        <v>373</v>
+      </c>
+      <c r="E39" t="s">
+        <v>83</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>383</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>64</v>
+      </c>
+      <c r="D41">
+        <v>370</v>
+      </c>
+      <c r="E41" t="s">
+        <v>83</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42">
+        <v>290</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>460</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44">
+        <v>373</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45">
+        <v>3493</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>250</v>
+      </c>
+      <c r="E46" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47">
+        <v>400</v>
+      </c>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>299</v>
+      </c>
+      <c r="E48" t="s">
+        <v>83</v>
+      </c>
+      <c r="F48" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>51</v>
+      </c>
+      <c r="D49">
+        <v>366</v>
+      </c>
+      <c r="E49" t="s">
+        <v>83</v>
+      </c>
+      <c r="F49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53">
+        <v>486</v>
+      </c>
+      <c r="E53" t="s">
+        <v>83</v>
+      </c>
+      <c r="F53" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54">
+        <v>692</v>
+      </c>
+      <c r="E54" t="s">
+        <v>83</v>
+      </c>
+      <c r="F54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>290</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56">
+        <v>1214</v>
+      </c>
+      <c r="E56" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>84</v>
+      </c>
+      <c r="B58">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58">
+        <v>3871</v>
+      </c>
+      <c r="E58" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>85</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>22</v>
+      </c>
+      <c r="D59">
+        <v>431</v>
+      </c>
+      <c r="E59" t="s">
+        <v>83</v>
+      </c>
+      <c r="F59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60">
+        <v>668</v>
+      </c>
+      <c r="E60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61">
+        <v>370</v>
+      </c>
+      <c r="E61" t="s">
+        <v>14</v>
+      </c>
+      <c r="F61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62">
+        <v>3</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>360</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63">
+        <v>16592</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64">
+        <v>250</v>
+      </c>
+      <c r="E64" t="s">
+        <v>14</v>
+      </c>
+      <c r="F64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65">
+        <v>606</v>
+      </c>
+      <c r="E65" t="s">
+        <v>14</v>
+      </c>
+      <c r="F65" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>290</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67">
+        <v>370</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>2067</v>
+      </c>
+      <c r="E68" t="s">
+        <v>14</v>
+      </c>
+      <c r="F68" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69">
+        <v>692</v>
+      </c>
+      <c r="E69" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70">
+        <v>383</v>
+      </c>
+      <c r="E70" t="s">
+        <v>14</v>
+      </c>
+      <c r="F70" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71">
+        <v>400</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72">
+        <v>250</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73">
+        <v>370</v>
+      </c>
+      <c r="E73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>2220</v>
+      </c>
+      <c r="E74" t="s">
+        <v>83</v>
+      </c>
+      <c r="F74" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>102</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75">
+        <v>400</v>
+      </c>
+      <c r="E75" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76">
+        <v>2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>66</v>
+      </c>
+      <c r="D76">
+        <v>290</v>
+      </c>
+      <c r="E76" t="s">
+        <v>14</v>
+      </c>
+      <c r="F76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77">
+        <v>1786</v>
+      </c>
+      <c r="E77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F77" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>105</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78">
+        <v>1222</v>
+      </c>
+      <c r="E78" t="s">
+        <v>83</v>
+      </c>
+      <c r="F78" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>106</v>
+      </c>
+      <c r="B79">
+        <v>2</v>
+      </c>
+      <c r="C79" t="s">
+        <v>51</v>
+      </c>
+      <c r="D79">
+        <v>2334</v>
+      </c>
+      <c r="E79" t="s">
+        <v>83</v>
+      </c>
+      <c r="F79" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80">
+        <v>280</v>
+      </c>
+      <c r="E80" t="s">
+        <v>14</v>
+      </c>
+      <c r="F80" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81">
+        <v>437</v>
+      </c>
+      <c r="E81" t="s">
+        <v>83</v>
+      </c>
+      <c r="F81" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82">
+        <v>370</v>
+      </c>
+      <c r="E82" t="s">
+        <v>14</v>
+      </c>
+      <c r="F82" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83">
+        <v>370</v>
+      </c>
+      <c r="E83" t="s">
+        <v>14</v>
+      </c>
+      <c r="F83" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84">
+        <v>2</v>
+      </c>
+      <c r="C84" t="s">
+        <v>40</v>
+      </c>
+      <c r="D84">
+        <v>310</v>
+      </c>
+      <c r="E84" t="s">
+        <v>14</v>
+      </c>
+      <c r="F84" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>22</v>
+      </c>
+      <c r="D85">
+        <v>570</v>
+      </c>
+      <c r="E85" t="s">
+        <v>83</v>
+      </c>
+      <c r="F85" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86">
+        <v>2</v>
+      </c>
+      <c r="C86" t="s">
+        <v>40</v>
+      </c>
+      <c r="D86">
+        <v>363</v>
+      </c>
+      <c r="E86" t="s">
+        <v>14</v>
+      </c>
+      <c r="F86" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>115</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>250</v>
+      </c>
+      <c r="E87" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>116</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>250</v>
+      </c>
+      <c r="E88" t="s">
+        <v>14</v>
+      </c>
+      <c r="F88" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>117</v>
+      </c>
+      <c r="B89">
+        <v>2</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89">
+        <v>360</v>
+      </c>
+      <c r="E89" t="s">
+        <v>14</v>
+      </c>
+      <c r="F89" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+      <c r="C90" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90">
+        <v>548</v>
+      </c>
+      <c r="E90" t="s">
+        <v>14</v>
+      </c>
+      <c r="F90" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>119</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>68</v>
+      </c>
+      <c r="D91">
+        <v>560</v>
+      </c>
+      <c r="E91" t="s">
+        <v>14</v>
+      </c>
+      <c r="F91" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92">
+        <v>250</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>121</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93">
+        <v>370</v>
+      </c>
+      <c r="E93" t="s">
+        <v>14</v>
+      </c>
+      <c r="F93" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+      <c r="C94" t="s">
+        <v>24</v>
+      </c>
+      <c r="D94">
+        <v>370</v>
+      </c>
+      <c r="E94" t="s">
+        <v>14</v>
+      </c>
+      <c r="F94" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>2780</v>
+      </c>
+      <c r="E95" t="s">
+        <v>14</v>
+      </c>
+      <c r="F95" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>14344</v>
+      </c>
+      <c r="E96" t="s">
+        <v>14</v>
+      </c>
+      <c r="F96" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>125</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>40</v>
+      </c>
+      <c r="D97">
+        <v>350</v>
+      </c>
+      <c r="E97" t="s">
+        <v>14</v>
+      </c>
+      <c r="F97" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>43</v>
+      </c>
+      <c r="D98">
+        <v>696</v>
+      </c>
+      <c r="E98" t="s">
+        <v>14</v>
+      </c>
+      <c r="F98" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>127</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>40</v>
+      </c>
+      <c r="D99">
+        <v>18762</v>
+      </c>
+      <c r="E99" t="s">
+        <v>14</v>
+      </c>
+      <c r="F99" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>128</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>495</v>
+      </c>
+      <c r="E100" t="s">
+        <v>14</v>
+      </c>
+      <c r="F100" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>129</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>48</v>
+      </c>
+      <c r="D101">
+        <v>560</v>
+      </c>
+      <c r="E101" t="s">
+        <v>14</v>
+      </c>
+      <c r="F101" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>130</v>
+      </c>
+      <c r="B102">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>43</v>
+      </c>
+      <c r="D102">
+        <v>435</v>
+      </c>
+      <c r="E102" t="s">
+        <v>14</v>
+      </c>
+      <c r="F102" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>131</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>280</v>
+      </c>
+      <c r="E103" t="s">
+        <v>14</v>
+      </c>
+      <c r="F103" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>132</v>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>3797</v>
+      </c>
+      <c r="E104" t="s">
+        <v>14</v>
+      </c>
+      <c r="F104" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>133</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105">
+        <v>422</v>
+      </c>
+      <c r="E105" t="s">
+        <v>14</v>
+      </c>
+      <c r="F105" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>134</v>
+      </c>
+      <c r="B106">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106">
+        <v>474</v>
+      </c>
+      <c r="E106" t="s">
+        <v>83</v>
+      </c>
+      <c r="F106" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>136</v>
+      </c>
+      <c r="B107">
+        <v>1</v>
+      </c>
+      <c r="C107" t="s">
+        <v>31</v>
+      </c>
+      <c r="D107">
+        <v>1243</v>
+      </c>
+      <c r="E107" t="s">
+        <v>14</v>
+      </c>
+      <c r="F107" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108">
+        <v>1</v>
+      </c>
+      <c r="C108" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108">
+        <v>370</v>
+      </c>
+      <c r="E108" t="s">
+        <v>14</v>
+      </c>
+      <c r="F108" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>138</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109">
+        <v>3765</v>
+      </c>
+      <c r="E109" t="s">
+        <v>14</v>
+      </c>
+      <c r="F109" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>139</v>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="s">
+        <v>26</v>
+      </c>
+      <c r="D110">
+        <v>4697</v>
+      </c>
+      <c r="E110" t="s">
+        <v>14</v>
+      </c>
+      <c r="F110" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111">
+        <v>370</v>
+      </c>
+      <c r="E111" t="s">
+        <v>14</v>
+      </c>
+      <c r="F111" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>141</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>66</v>
+      </c>
+      <c r="D112">
+        <v>290</v>
+      </c>
+      <c r="E112" t="s">
+        <v>14</v>
+      </c>
+      <c r="F112" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>40</v>
+      </c>
+      <c r="D113">
+        <v>403</v>
+      </c>
+      <c r="E113" t="s">
+        <v>14</v>
+      </c>
+      <c r="F113" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114">
+        <v>166</v>
+      </c>
+      <c r="E114" t="s">
+        <v>83</v>
+      </c>
+      <c r="F114" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>43</v>
+      </c>
+      <c r="D115">
+        <v>513</v>
+      </c>
+      <c r="E115" t="s">
+        <v>14</v>
+      </c>
+      <c r="F115" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116">
+        <v>511</v>
+      </c>
+      <c r="E116" t="s">
+        <v>14</v>
+      </c>
+      <c r="F116" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117">
+        <v>3</v>
+      </c>
+      <c r="C117" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117">
+        <v>280</v>
+      </c>
+      <c r="E117" t="s">
+        <v>14</v>
+      </c>
+      <c r="F117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118">
+        <v>3</v>
+      </c>
+      <c r="C118" t="s">
+        <v>148</v>
+      </c>
+      <c r="D118">
+        <v>250</v>
+      </c>
+      <c r="E118" t="s">
+        <v>14</v>
+      </c>
+      <c r="F118" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>149</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>48</v>
+      </c>
+      <c r="D119">
+        <v>3751</v>
+      </c>
+      <c r="E119" t="s">
+        <v>14</v>
+      </c>
+      <c r="F119" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>150</v>
+      </c>
+      <c r="B120">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D120">
+        <v>2050</v>
+      </c>
+      <c r="E120" t="s">
+        <v>14</v>
+      </c>
+      <c r="F120" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>151</v>
+      </c>
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>1798</v>
+      </c>
+      <c r="E121" t="s">
+        <v>14</v>
+      </c>
+      <c r="F121" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>1</v>
+      </c>
+      <c r="C122" t="s">
+        <v>31</v>
+      </c>
+      <c r="D122">
+        <v>1253</v>
+      </c>
+      <c r="E122" t="s">
+        <v>14</v>
+      </c>
+      <c r="F122" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>153</v>
+      </c>
+      <c r="B123">
+        <v>3</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123">
+        <v>1223</v>
+      </c>
+      <c r="E123" t="s">
+        <v>14</v>
+      </c>
+      <c r="F123" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>154</v>
+      </c>
+      <c r="B124">
+        <v>1</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+      <c r="D124">
+        <v>370</v>
+      </c>
+      <c r="E124" t="s">
+        <v>14</v>
+      </c>
+      <c r="F124" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125" t="s">
+        <v>7</v>
+      </c>
+      <c r="D125">
+        <v>262</v>
+      </c>
+      <c r="E125" t="s">
+        <v>83</v>
+      </c>
+      <c r="F125" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore: 달란트 일일 백업 (2026-10-25)
</commit_message>
<xml_diff>
--- a/backup/talents_backup.xlsx
+++ b/backup/talents_backup.xlsx
@@ -44,13 +44,14 @@
     <sheet sheetId="38" name="2026-10-22" state="visible" r:id="rId41"/>
     <sheet sheetId="39" name="2026-10-23" state="visible" r:id="rId42"/>
     <sheet sheetId="40" name="2026-10-24" state="visible" r:id="rId43"/>
+    <sheet sheetId="41" name="2026-10-25" state="visible" r:id="rId44"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20036" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20538" uniqueCount="157">
   <si>
     <t>이름</t>
   </si>
@@ -88900,6 +88901,2525 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F125"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>394</v>
+      </c>
+      <c r="E2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>783</v>
+      </c>
+      <c r="E3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>21959</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>18657</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>350</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>323</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>520</v>
+      </c>
+      <c r="E8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9">
+        <v>370</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>360</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>250</v>
+      </c>
+      <c r="E12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <v>303</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14">
+        <v>945</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15">
+        <v>10362</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16">
+        <v>226</v>
+      </c>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>280</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>350</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>360</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>703</v>
+      </c>
+      <c r="E20" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>310</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>647</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23">
+        <v>420</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24">
+        <v>370</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      